<commit_message>
Updates of previously existing templates and examples after an internal consistency check. Addition of new templates and examples. Updated lookup table to account for a new artifact, and document manifest updated to reflect added templates and examples. 50 templates and examples [of the library of 163] are complete and included here.
</commit_message>
<xml_diff>
--- a/public/templates/examples/A-009-RiskRegister-EXAMPLE-L.xlsx
+++ b/public/templates/examples/A-009-RiskRegister-EXAMPLE-L.xlsx
@@ -330,17 +330,17 @@
     </font>
     <font>
       <sz val="10"/>
-      <name val="Arial"/>
+      <name val="Aptos"/>
       <family val="0"/>
     </font>
     <font>
       <sz val="10"/>
-      <name val="Arial"/>
+      <name val="Aptos"/>
       <family val="0"/>
     </font>
     <font>
       <sz val="10"/>
-      <name val="Arial"/>
+      <name val="Aptos"/>
       <family val="0"/>
     </font>
     <font>

</xml_diff>